<commit_message>
Update P2P Dashboard with data up to March 18, 2026
- Replaced Excel source files with updated versions from GitHub.
- Regenerated p2p_data.parquet to include 197 new rows from March 2026.
- Verified final max PO date is 2026-03-18.
- Cleaned up repository junk files (__pycache__).

Co-authored-by: Pauriktrivedi <96005961+Pauriktrivedi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MLPL.xlsx
+++ b/MLPL.xlsx
@@ -240,7 +240,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">03-03-2026 05:03:22
+            <t xml:space="preserve">18-03-2026 16:39:15
 </t>
           </r>
           <r>
@@ -289,7 +289,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">28-02-2026</t>
+            <t xml:space="preserve">18-03-2026</t>
           </r>
         </is>
       </c>
@@ -1397,11 +1397,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG7">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00004</t>
+          <t xml:space="preserve">ML/PO/25-26/00019</t>
         </is>
       </c>
       <c s="4" r="AH7">
-        <v>45810.7549884259</v>
+        <v>46098.4664583333</v>
       </c>
       <c s="3" t="inlineStr" r="AI7">
         <is>
@@ -1581,11 +1581,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG8">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00004</t>
+          <t xml:space="preserve">ML/PO/25-26/00019</t>
         </is>
       </c>
       <c s="4" r="AH8">
-        <v>45810.7549884259</v>
+        <v>46098.4664583333</v>
       </c>
       <c s="3" t="inlineStr" r="AI8">
         <is>
@@ -1771,13 +1771,15 @@
       </c>
       <c s="3" t="inlineStr" r="AG9">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="AH9"/>
+          <t xml:space="preserve">ML/PO/25-26/00019</t>
+        </is>
+      </c>
+      <c s="4" r="AH9">
+        <v>46098.4664583333</v>
+      </c>
       <c s="3" t="inlineStr" r="AI9">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FIREFLINK PRIVATE LIMITED</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AJ9">
@@ -2896,11 +2898,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG15">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH15">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI15">
         <is>
@@ -3086,11 +3088,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG16">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH16">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI16">
         <is>
@@ -3277,11 +3279,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG17">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH17">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI17">
         <is>
@@ -3467,11 +3469,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG18">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH18">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI18">
         <is>
@@ -3657,11 +3659,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG19">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH19">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI19">
         <is>
@@ -3847,11 +3849,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG20">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH20">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI20">
         <is>
@@ -4037,11 +4039,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG21">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH21">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI21">
         <is>
@@ -4227,11 +4229,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG22">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH22">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI22">
         <is>
@@ -4417,11 +4419,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG23">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH23">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI23">
         <is>
@@ -4607,11 +4609,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG24">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH24">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI24">
         <is>
@@ -4798,11 +4800,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG25">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH25">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI25">
         <is>
@@ -5368,11 +5370,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG28">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH28">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI28">
         <is>
@@ -5558,11 +5560,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG29">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH29">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI29">
         <is>
@@ -5748,11 +5750,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG30">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH30">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI30">
         <is>
@@ -6506,11 +6508,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG34">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH34">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI34">
         <is>
@@ -6696,11 +6698,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG35">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH35">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI35">
         <is>
@@ -7074,11 +7076,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG37">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH37">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI37">
         <is>
@@ -7264,11 +7266,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG38">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH38">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI38">
         <is>
@@ -7454,11 +7456,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG39">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH39">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI39">
         <is>
@@ -7834,11 +7836,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG41">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH41">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI41">
         <is>
@@ -8784,11 +8786,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG46">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH46">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI46">
         <is>
@@ -9354,11 +9356,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG49">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH49">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI49">
         <is>
@@ -9544,11 +9546,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG50">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH50">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI50">
         <is>
@@ -9734,11 +9736,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG51">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH51">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI51">
         <is>
@@ -9924,11 +9926,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG52">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH52">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI52">
         <is>
@@ -10115,11 +10117,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG53">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00007</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH53">
-        <v>45832.7777662037</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI53">
         <is>
@@ -10875,11 +10877,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG57">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH57">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI57">
         <is>
@@ -11253,11 +11255,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG59">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH59">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI59">
         <is>
@@ -11443,11 +11445,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG60">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH60">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI60">
         <is>
@@ -11822,11 +11824,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG62">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH62">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI62">
         <is>
@@ -12012,11 +12014,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG63">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH63">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI63">
         <is>
@@ -12958,11 +12960,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG68">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH68">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI68">
         <is>
@@ -13148,11 +13150,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG69">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH69">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI69">
         <is>
@@ -13338,11 +13340,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG70">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00007</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH70">
-        <v>45832.7777662037</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI70">
         <is>
@@ -13528,11 +13530,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG71">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH71">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI71">
         <is>
@@ -13718,11 +13720,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG72">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH72">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI72">
         <is>
@@ -14098,11 +14100,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG74">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00007</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH74">
-        <v>45832.7777662037</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI74">
         <is>
@@ -15048,11 +15050,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG79">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH79">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI79">
         <is>
@@ -15238,11 +15240,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG80">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH80">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI80">
         <is>
@@ -16762,11 +16764,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG88">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH88">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI88">
         <is>
@@ -16952,11 +16954,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG89">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH89">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI89">
         <is>
@@ -17522,11 +17524,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG92">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH92">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI92">
         <is>
@@ -17712,11 +17714,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG93">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH93">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI93">
         <is>
@@ -18281,11 +18283,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG96">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH96">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI96">
         <is>
@@ -18471,11 +18473,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG97">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH97">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI97">
         <is>
@@ -18851,11 +18853,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG99">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH99">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI99">
         <is>
@@ -19041,11 +19043,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG100">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH100">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI100">
         <is>
@@ -19611,11 +19613,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG103">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00016</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH103">
-        <v>45929.5327199074</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI103">
         <is>
@@ -24136,11 +24138,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG127">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH127">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI127">
         <is>
@@ -24326,11 +24328,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG128">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH128">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI128">
         <is>
@@ -24516,11 +24518,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG129">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH129">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI129">
         <is>
@@ -24706,11 +24708,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG130">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH130">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI130">
         <is>
@@ -25086,11 +25088,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG132">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH132">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI132">
         <is>
@@ -25465,11 +25467,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG134">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH134">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI134">
         <is>
@@ -26034,11 +26036,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG137">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH137">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI137">
         <is>
@@ -26224,11 +26226,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG138">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH138">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI138">
         <is>
@@ -26414,11 +26416,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG139">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH139">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI139">
         <is>
@@ -27174,11 +27176,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG143">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH143">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI143">
         <is>
@@ -27364,11 +27366,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG144">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH144">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI144">
         <is>
@@ -27933,11 +27935,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG147">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH147">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI147">
         <is>
@@ -28123,11 +28125,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG148">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH148">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI148">
         <is>
@@ -28693,11 +28695,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG151">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00012</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH151">
-        <v>45833.5999652778</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI151">
         <is>
@@ -28883,11 +28885,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG152">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH152">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI152">
         <is>
@@ -29073,11 +29075,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG153">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH153">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI153">
         <is>
@@ -29263,11 +29265,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG154">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH154">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI154">
         <is>
@@ -29453,11 +29455,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG155">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH155">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI155">
         <is>
@@ -29833,11 +29835,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG157">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH157">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI157">
         <is>
@@ -30023,11 +30025,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG158">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH158">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI158">
         <is>
@@ -30403,11 +30405,11 @@
       </c>
       <c s="3" t="inlineStr" r="AG160">
         <is>
-          <t xml:space="preserve">ML/PO/25-26/00013</t>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
         </is>
       </c>
       <c s="4" r="AH160">
-        <v>45833.6977893518</v>
+        <v>46087.7545601852</v>
       </c>
       <c s="3" t="inlineStr" r="AI160">
         <is>
@@ -30543,36 +30545,42 @@
       </c>
       <c s="9" t="inlineStr" r="T161">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U161">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V161"/>
-      <c s="3" t="str" r="W161"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V161">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W161">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X161">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y161">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z161">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="8" r="AA161">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="9" t="inlineStr" r="AB161">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC161"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC161">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD161">
         <v>0</v>
       </c>
@@ -30581,7 +30589,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF161">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG161">
@@ -30609,12 +30617,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL161">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM161">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN161">
@@ -30634,7 +30642,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ161">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -30726,36 +30734,42 @@
       </c>
       <c s="9" t="inlineStr" r="T162">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U162">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V162"/>
-      <c s="3" t="str" r="W162"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V162">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W162">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X162">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y162">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z162">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="8" r="AA162">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="9" t="inlineStr" r="AB162">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC162"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC162">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD162">
         <v>0</v>
       </c>
@@ -30764,7 +30778,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF162">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG162">
@@ -30792,12 +30806,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL162">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM162">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN162">
@@ -30817,7 +30831,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ162">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -30909,36 +30923,42 @@
       </c>
       <c s="9" t="inlineStr" r="T163">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U163">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V163"/>
-      <c s="3" t="str" r="W163"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V163">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W163">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X163">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y163">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z163">
-        <v>0</v>
+        <v>122500</v>
       </c>
       <c s="8" r="AA163">
-        <v>0</v>
+        <v>122500</v>
       </c>
       <c s="9" t="inlineStr" r="AB163">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC163"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC163">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD163">
         <v>0</v>
       </c>
@@ -30947,7 +30967,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF163">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG163">
@@ -30975,12 +30995,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL163">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM163">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN163">
@@ -31000,7 +31020,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ163">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -31092,36 +31112,42 @@
       </c>
       <c s="9" t="inlineStr" r="T164">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U164">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V164"/>
-      <c s="3" t="str" r="W164"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V164">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W164">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X164">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y164">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z164">
-        <v>0</v>
+        <v>148750</v>
       </c>
       <c s="8" r="AA164">
-        <v>0</v>
+        <v>148750</v>
       </c>
       <c s="9" t="inlineStr" r="AB164">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC164"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC164">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD164">
         <v>0</v>
       </c>
@@ -31130,7 +31156,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF164">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG164">
@@ -31158,12 +31184,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL164">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM164">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN164">
@@ -31183,7 +31209,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ164">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -31275,36 +31301,42 @@
       </c>
       <c s="9" t="inlineStr" r="T165">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U165">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V165"/>
-      <c s="3" t="str" r="W165"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V165">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W165">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X165">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y165">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z165">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="8" r="AA165">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="9" t="inlineStr" r="AB165">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC165"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC165">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD165">
         <v>0</v>
       </c>
@@ -31313,7 +31345,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF165">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG165">
@@ -31341,12 +31373,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL165">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM165">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN165">
@@ -31366,7 +31398,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ165">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -31458,36 +31490,42 @@
       </c>
       <c s="9" t="inlineStr" r="T166">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U166">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V166"/>
-      <c s="3" t="str" r="W166"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V166">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W166">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X166">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y166">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z166">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="8" r="AA166">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="9" t="inlineStr" r="AB166">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC166"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC166">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD166">
         <v>0</v>
       </c>
@@ -31496,7 +31534,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF166">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG166">
@@ -31524,12 +31562,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL166">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM166">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN166">
@@ -31549,7 +31587,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ166">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -31641,36 +31679,42 @@
       </c>
       <c s="9" t="inlineStr" r="T167">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U167">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V167"/>
-      <c s="3" t="str" r="W167"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V167">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W167">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X167">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y167">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z167">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="8" r="AA167">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="9" t="inlineStr" r="AB167">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC167"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC167">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD167">
         <v>0</v>
       </c>
@@ -31679,7 +31723,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF167">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG167">
@@ -31707,12 +31751,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL167">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM167">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN167">
@@ -31732,7 +31776,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ167">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -31824,36 +31868,42 @@
       </c>
       <c s="9" t="inlineStr" r="T168">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U168">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V168"/>
-      <c s="3" t="str" r="W168"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V168">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W168">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X168">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y168">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z168">
-        <v>0</v>
+        <v>70291.67</v>
       </c>
       <c s="8" r="AA168">
-        <v>0</v>
+        <v>70291.67</v>
       </c>
       <c s="9" t="inlineStr" r="AB168">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC168"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC168">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD168">
         <v>0</v>
       </c>
@@ -31862,7 +31912,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF168">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG168">
@@ -31890,12 +31940,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL168">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM168">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN168">
@@ -31915,7 +31965,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ168">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32007,36 +32057,42 @@
       </c>
       <c s="9" t="inlineStr" r="T169">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U169">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V169"/>
-      <c s="3" t="str" r="W169"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V169">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W169">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X169">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y169">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z169">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="8" r="AA169">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="9" t="inlineStr" r="AB169">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC169"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC169">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD169">
         <v>0</v>
       </c>
@@ -32045,7 +32101,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF169">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG169">
@@ -32073,12 +32129,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL169">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM169">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN169">
@@ -32098,7 +32154,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ169">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32190,36 +32246,42 @@
       </c>
       <c s="9" t="inlineStr" r="T170">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U170">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V170"/>
-      <c s="3" t="str" r="W170"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V170">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W170">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X170">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y170">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z170">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="8" r="AA170">
-        <v>0</v>
+        <v>74375</v>
       </c>
       <c s="9" t="inlineStr" r="AB170">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC170"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC170">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD170">
         <v>0</v>
       </c>
@@ -32228,7 +32290,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF170">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG170">
@@ -32256,12 +32318,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL170">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM170">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN170">
@@ -32281,7 +32343,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ170">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32373,36 +32435,42 @@
       </c>
       <c s="9" t="inlineStr" r="T171">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U171">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V171"/>
-      <c s="3" t="str" r="W171"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V171">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W171">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X171">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y171">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z171">
-        <v>0</v>
+        <v>70291.67</v>
       </c>
       <c s="8" r="AA171">
-        <v>0</v>
+        <v>70291.67</v>
       </c>
       <c s="9" t="inlineStr" r="AB171">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC171"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC171">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD171">
         <v>0</v>
       </c>
@@ -32411,7 +32479,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF171">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG171">
@@ -32439,12 +32507,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL171">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM171">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN171">
@@ -32464,7 +32532,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ171">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32558,36 +32626,42 @@
       </c>
       <c s="9" t="inlineStr" r="T172">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U172">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V172"/>
-      <c s="3" t="str" r="W172"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V172">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W172">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X172">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y172">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z172">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="8" r="AA172">
-        <v>0</v>
+        <v>49145.83</v>
       </c>
       <c s="9" t="inlineStr" r="AB172">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC172"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC172">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD172">
         <v>0</v>
       </c>
@@ -32596,7 +32670,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF172">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG172">
@@ -32624,12 +32698,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL172">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM172">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN172">
@@ -32649,7 +32723,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ172">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32741,36 +32815,42 @@
       </c>
       <c s="9" t="inlineStr" r="T173">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U173">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V173"/>
-      <c s="3" t="str" r="W173"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V173">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W173">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X173">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y173">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z173">
-        <v>0</v>
+        <v>30187.5</v>
       </c>
       <c s="8" r="AA173">
-        <v>0</v>
+        <v>30187.5</v>
       </c>
       <c s="9" t="inlineStr" r="AB173">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC173"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC173">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD173">
         <v>0</v>
       </c>
@@ -32779,7 +32859,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF173">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG173">
@@ -32807,12 +32887,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL173">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM173">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN173">
@@ -32832,7 +32912,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ173">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -32924,36 +33004,42 @@
       </c>
       <c s="9" t="inlineStr" r="T174">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U174">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V174"/>
-      <c s="3" t="str" r="W174"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V174">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W174">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X174">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y174">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z174">
-        <v>0</v>
+        <v>24587.5</v>
       </c>
       <c s="8" r="AA174">
-        <v>0</v>
+        <v>24587.5</v>
       </c>
       <c s="9" t="inlineStr" r="AB174">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC174"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC174">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD174">
         <v>0</v>
       </c>
@@ -32962,7 +33048,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF174">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG174">
@@ -32990,12 +33076,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL174">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM174">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN174">
@@ -33015,7 +33101,7 @@
       </c>
       <c s="3" t="inlineStr" r="AQ174">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
@@ -33107,36 +33193,42 @@
       </c>
       <c s="9" t="inlineStr" r="T175">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U175">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V175"/>
-      <c s="3" t="str" r="W175"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V175">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W175">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X175">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y175">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z175">
-        <v>0</v>
+        <v>55270.83</v>
       </c>
       <c s="8" r="AA175">
-        <v>0</v>
+        <v>55270.83</v>
       </c>
       <c s="9" t="inlineStr" r="AB175">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC175"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC175">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD175">
         <v>0</v>
       </c>
@@ -33145,7 +33237,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF175">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG175">
@@ -33173,12 +33265,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL175">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM175">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN175">
@@ -33198,11 +33290,11 @@
       </c>
       <c s="3" t="inlineStr" r="AQ175">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
-    <row r="176" ht="12.2" customHeight="0">
+    <row r="176" ht="12.25" customHeight="0">
       <c s="3" t="inlineStr" r="A176">
         <is>
           <t xml:space="preserve">PR004319</t>
@@ -33290,36 +33382,42 @@
       </c>
       <c s="9" t="inlineStr" r="T176">
         <is>
-          <t xml:space="preserve">InReview</t>
+          <t xml:space="preserve">Closed</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="U176">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="3" t="str" r="V176"/>
-      <c s="3" t="str" r="W176"/>
+          <t xml:space="preserve">ML/PO/25-26/00018</t>
+        </is>
+      </c>
+      <c s="4" r="V176">
+        <v>46087.7545601852</v>
+      </c>
+      <c s="4" r="W176">
+        <v>46087</v>
+      </c>
       <c s="3" t="inlineStr" r="X176">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MathWorks India Private Limited</t>
         </is>
       </c>
       <c s="6" r="Y176">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c s="7" r="Z176">
-        <v>0</v>
+        <v>51479.17</v>
       </c>
       <c s="8" r="AA176">
-        <v>0</v>
+        <v>51479.17</v>
       </c>
       <c s="9" t="inlineStr" r="AB176">
         <is>
-          <t xml:space="preserve">None</t>
-        </is>
-      </c>
-      <c s="3" t="str" r="AC176"/>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="4" r="AC176">
+        <v>46093.309537037</v>
+      </c>
       <c s="6" r="AD176">
         <v>0</v>
       </c>
@@ -33328,7 +33426,7 @@
       </c>
       <c s="3" t="inlineStr" r="AF176">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MMW2425154</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AG176">
@@ -33356,12 +33454,12 @@
       </c>
       <c s="3" t="inlineStr" r="AL176">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ML.SFL.MTLB</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AM176">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Software Licence- Matlab</t>
         </is>
       </c>
       <c s="3" t="inlineStr" r="AN176">
@@ -33381,11 +33479,385 @@
       </c>
       <c s="3" t="inlineStr" r="AQ176">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">00000321</t>
         </is>
       </c>
     </row>
-    <row r="177" ht="0.05" customHeight="1"/>
+    <row r="177" ht="12.25" customHeight="0">
+      <c s="3" t="inlineStr" r="A177">
+        <is>
+          <t xml:space="preserve">PR004385</t>
+        </is>
+      </c>
+      <c s="4" r="B177">
+        <v>46097.7151041667</v>
+      </c>
+      <c s="3" t="inlineStr" r="C177">
+        <is>
+          <t xml:space="preserve">ML : Fireflink Pricing Details – User-Based Licensing (NR)</t>
+        </is>
+      </c>
+      <c s="5" r="D177">
+        <v>1</v>
+      </c>
+      <c s="3" t="inlineStr" r="E177">
+        <is>
+          <t xml:space="preserve">BG16</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="F177">
+        <is>
+          <t xml:space="preserve">MMW2223268</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="G177">
+        <is>
+          <t xml:space="preserve">Service</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="H177">
+        <is>
+          <t xml:space="preserve">SER_1339</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="I177">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="J177">
+        <is>
+          <t xml:space="preserve">FireFlink Extreme Automation Platform (Cloud Basic)</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="K177">
+        <is>
+          <t xml:space="preserve">FireFlink Extreme Automation Platform (Cloud Basic). Automated Software Testing Platform for Web, Android, iOS and APIs
+</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="L177">
+        <is>
+          <t xml:space="preserve">MATTERLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="M177">
+        <is>
+          <t xml:space="preserve">MLNK01</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="N177">
+        <is>
+          <t xml:space="preserve">MLWH</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="O177">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" r="P177">
+        <v>3</v>
+      </c>
+      <c s="3" t="inlineStr" r="Q177">
+        <is>
+          <t xml:space="preserve">INR</t>
+        </is>
+      </c>
+      <c s="7" r="R177">
+        <v>23081.85</v>
+      </c>
+      <c s="8" r="S177">
+        <v>69245.55</v>
+      </c>
+      <c s="9" t="inlineStr" r="T177">
+        <is>
+          <t xml:space="preserve">Closed</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="U177">
+        <is>
+          <t xml:space="preserve">ML/PO/25-26/00019</t>
+        </is>
+      </c>
+      <c s="4" r="V177">
+        <v>46098.4664583333</v>
+      </c>
+      <c s="4" r="W177">
+        <v>46098</v>
+      </c>
+      <c s="3" t="inlineStr" r="X177">
+        <is>
+          <t xml:space="preserve">FIREFLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="6" r="Y177">
+        <v>3</v>
+      </c>
+      <c s="7" r="Z177">
+        <v>20715</v>
+      </c>
+      <c s="8" r="AA177">
+        <v>62145</v>
+      </c>
+      <c s="9" t="inlineStr" r="AB177">
+        <is>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="3" t="str" r="AC177"/>
+      <c s="6" r="AD177">
+        <v>0</v>
+      </c>
+      <c s="6" r="AE177">
+        <v>0</v>
+      </c>
+      <c s="3" t="inlineStr" r="AF177">
+        <is>
+          <t xml:space="preserve">MMW2425154</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AG177">
+        <is>
+          <t xml:space="preserve">ML/PO/25-26/00004</t>
+        </is>
+      </c>
+      <c s="4" r="AH177">
+        <v>45810.7549884259</v>
+      </c>
+      <c s="3" t="inlineStr" r="AI177">
+        <is>
+          <t xml:space="preserve">FIREFLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AJ177">
+        <is>
+          <t xml:space="preserve">ML.DT.SFL.CFL</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AK177">
+        <is>
+          <t xml:space="preserve">Firelink Cloud</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AL177">
+        <is>
+          <t xml:space="preserve">ML.DT.SFL.CFL</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AM177">
+        <is>
+          <t xml:space="preserve">Firelink Cloud</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AN177">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AO177">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AP177">
+        <is>
+          <t xml:space="preserve">00000381</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AQ177">
+        <is>
+          <t xml:space="preserve">00000381</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="12.2" customHeight="0">
+      <c s="3" t="inlineStr" r="A178">
+        <is>
+          <t xml:space="preserve">PR004385</t>
+        </is>
+      </c>
+      <c s="4" r="B178">
+        <v>46097.7151041667</v>
+      </c>
+      <c s="3" t="inlineStr" r="C178">
+        <is>
+          <t xml:space="preserve">ML : Fireflink Pricing Details – User-Based Licensing (NR)</t>
+        </is>
+      </c>
+      <c s="5" r="D178">
+        <v>2</v>
+      </c>
+      <c s="3" t="inlineStr" r="E178">
+        <is>
+          <t xml:space="preserve">BG16</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="F178">
+        <is>
+          <t xml:space="preserve">MMW2223268</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="G178">
+        <is>
+          <t xml:space="preserve">Service</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="H178">
+        <is>
+          <t xml:space="preserve">SER_2035</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="I178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="J178">
+        <is>
+          <t xml:space="preserve">FireFlink Cloud Mobile Testing Subscription</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="K178">
+        <is>
+          <t xml:space="preserve">Online device farm for Android and iOS devices for performing automation testing of mobile web applications and mobile apps
+</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="L178">
+        <is>
+          <t xml:space="preserve">MATTERLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="M178">
+        <is>
+          <t xml:space="preserve">MLNK01</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="N178">
+        <is>
+          <t xml:space="preserve">MLWH</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="O178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" r="P178">
+        <v>3</v>
+      </c>
+      <c s="3" t="inlineStr" r="Q178">
+        <is>
+          <t xml:space="preserve">INR</t>
+        </is>
+      </c>
+      <c s="7" r="R178">
+        <v>18373.15</v>
+      </c>
+      <c s="8" r="S178">
+        <v>55119.45</v>
+      </c>
+      <c s="9" t="inlineStr" r="T178">
+        <is>
+          <t xml:space="preserve">Closed</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="U178">
+        <is>
+          <t xml:space="preserve">ML/PO/25-26/00019</t>
+        </is>
+      </c>
+      <c s="4" r="V178">
+        <v>46098.4664583333</v>
+      </c>
+      <c s="4" r="W178">
+        <v>46098</v>
+      </c>
+      <c s="3" t="inlineStr" r="X178">
+        <is>
+          <t xml:space="preserve">FIREFLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="6" r="Y178">
+        <v>3</v>
+      </c>
+      <c s="7" r="Z178">
+        <v>15191</v>
+      </c>
+      <c s="8" r="AA178">
+        <v>45573</v>
+      </c>
+      <c s="9" t="inlineStr" r="AB178">
+        <is>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="3" t="str" r="AC178"/>
+      <c s="6" r="AD178">
+        <v>0</v>
+      </c>
+      <c s="6" r="AE178">
+        <v>0</v>
+      </c>
+      <c s="3" t="inlineStr" r="AF178">
+        <is>
+          <t xml:space="preserve">MMW2425154</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AG178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="str" r="AH178"/>
+      <c s="3" t="inlineStr" r="AI178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AJ178">
+        <is>
+          <t xml:space="preserve">ML.DT.SFL.CFL</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AK178">
+        <is>
+          <t xml:space="preserve">Firelink Cloud</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AL178">
+        <is>
+          <t xml:space="preserve">ML.DT.SFL.CFL</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AM178">
+        <is>
+          <t xml:space="preserve">Firelink Cloud</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AN178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AO178">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AP178">
+        <is>
+          <t xml:space="preserve">00000381</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AQ178">
+        <is>
+          <t xml:space="preserve">00000381</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:AS1"/>

</xml_diff>

<commit_message>
Update P2P dashboard with March 2026 data and stability improvements
- Integrated new Excel data files (MEPL, MLPL, MMPL, MMW) with data up to March 31, 2026.
- Regenerated p2p_data.parquet to reflect the latest records.
- Maintained stability fixes to prevent "Oh no" crashes (cache limits, session state optimization).
- preserved hierarchical Buyer Type logic and 'Gujarat' as default state for vendors.
- Verified dashboard rendering and data integrity.

Co-authored-by: Pauriktrivedi <96005961+Pauriktrivedi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MLPL.xlsx
+++ b/MLPL.xlsx
@@ -240,7 +240,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">18-03-2026 16:39:15
+            <t xml:space="preserve">31-03-2026 10:21:57
 </t>
           </r>
           <r>
@@ -289,7 +289,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">18-03-2026</t>
+            <t xml:space="preserve">31-03-2026</t>
           </r>
         </is>
       </c>
@@ -33605,7 +33605,9 @@
           <t xml:space="preserve">Backorder</t>
         </is>
       </c>
-      <c s="3" t="str" r="AC177"/>
+      <c s="4" r="AC177">
+        <v>46101.8442361111</v>
+      </c>
       <c s="6" r="AD177">
         <v>0</v>
       </c>
@@ -33671,7 +33673,7 @@
         </is>
       </c>
     </row>
-    <row r="178" ht="12.2" customHeight="0">
+    <row r="178" ht="12.25" customHeight="0">
       <c s="3" t="inlineStr" r="A178">
         <is>
           <t xml:space="preserve">PR004385</t>
@@ -33793,7 +33795,9 @@
           <t xml:space="preserve">Backorder</t>
         </is>
       </c>
-      <c s="3" t="str" r="AC178"/>
+      <c s="4" r="AC178">
+        <v>46101.8442361111</v>
+      </c>
       <c s="6" r="AD178">
         <v>0</v>
       </c>
@@ -33857,7 +33861,193 @@
         </is>
       </c>
     </row>
-    <row r="179" ht="0.05" customHeight="1"/>
+    <row r="179" ht="12.2" customHeight="0">
+      <c s="3" t="inlineStr" r="A179">
+        <is>
+          <t xml:space="preserve">PR004414</t>
+        </is>
+      </c>
+      <c s="4" r="B179">
+        <v>46105.7780902778</v>
+      </c>
+      <c s="3" t="inlineStr" r="C179">
+        <is>
+          <t xml:space="preserve">ML : Consultancy charge (Operations)</t>
+        </is>
+      </c>
+      <c s="5" r="D179">
+        <v>1</v>
+      </c>
+      <c s="3" t="inlineStr" r="E179">
+        <is>
+          <t xml:space="preserve">BG16</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="F179">
+        <is>
+          <t xml:space="preserve">MMW2223268</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="G179">
+        <is>
+          <t xml:space="preserve">Service</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="H179">
+        <is>
+          <t xml:space="preserve">SER_0844</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="I179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="J179">
+        <is>
+          <t xml:space="preserve">Consultancy charge</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="K179">
+        <is>
+          <t xml:space="preserve">Consultancy Charge 
+</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="L179">
+        <is>
+          <t xml:space="preserve">MATTERLINK PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="M179">
+        <is>
+          <t xml:space="preserve">MLNK01</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="N179">
+        <is>
+          <t xml:space="preserve">MLWH</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="O179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" r="P179">
+        <v>4</v>
+      </c>
+      <c s="3" t="inlineStr" r="Q179">
+        <is>
+          <t xml:space="preserve">INR</t>
+        </is>
+      </c>
+      <c s="7" r="R179">
+        <v>350000</v>
+      </c>
+      <c s="8" r="S179">
+        <v>1400000</v>
+      </c>
+      <c s="9" t="inlineStr" r="T179">
+        <is>
+          <t xml:space="preserve">Closed</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="U179">
+        <is>
+          <t xml:space="preserve">ML/PO/25-26/00020</t>
+        </is>
+      </c>
+      <c s="4" r="V179">
+        <v>46108.5190393518</v>
+      </c>
+      <c s="4" r="W179">
+        <v>46108</v>
+      </c>
+      <c s="3" t="inlineStr" r="X179">
+        <is>
+          <t xml:space="preserve">Sane Sai Charan</t>
+        </is>
+      </c>
+      <c s="6" r="Y179">
+        <v>4</v>
+      </c>
+      <c s="7" r="Z179">
+        <v>350000</v>
+      </c>
+      <c s="8" r="AA179">
+        <v>1400000</v>
+      </c>
+      <c s="9" t="inlineStr" r="AB179">
+        <is>
+          <t xml:space="preserve">Backorder</t>
+        </is>
+      </c>
+      <c s="3" t="str" r="AC179"/>
+      <c s="6" r="AD179">
+        <v>0</v>
+      </c>
+      <c s="6" r="AE179">
+        <v>0</v>
+      </c>
+      <c s="3" t="inlineStr" r="AF179">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AG179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="str" r="AH179"/>
+      <c s="3" t="inlineStr" r="AI179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AJ179">
+        <is>
+          <t xml:space="preserve">ML.G&amp;A.HR.CNST</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AK179">
+        <is>
+          <t xml:space="preserve">Consultant Link</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AL179">
+        <is>
+          <t xml:space="preserve">ML.G&amp;A.HR.CNST</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AM179">
+        <is>
+          <t xml:space="preserve">Consultant Link</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AN179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AO179">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AP179">
+        <is>
+          <t xml:space="preserve">00000641</t>
+        </is>
+      </c>
+      <c s="3" t="inlineStr" r="AQ179">
+        <is>
+          <t xml:space="preserve">00000641</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:AS1"/>

</xml_diff>